<commit_message>
Enhance functionality and improve data handling
This commit introduces several key updates across multiple files:

1. Added a new `orderDate` parameter to `GetSupplierDetail` for flexible data retrieval and filtering.
2. Implemented conditional logic to handle scenarios based on the presence of new parameters.
3. Updated database context usage to improve data access efficiency.
4. Enhanced error handling by throwing exceptions when expected data is not found.
5. Improved JavaScript functions with asynchronous handling for better user experience.
6. Updated configuration files to use more secure database access methods.
7. Added new entries to data import files to keep application data current.

These changes collectively enhance the application's performance, security, and user experience.
</commit_message>
<xml_diff>
--- a/wwwroot/file_temp/IMPORT_TRIAL.xlsx
+++ b/wwwroot/file_temp/IMPORT_TRIAL.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\20234111\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25F9C07-E7BB-41DA-8E59-E2203757C24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="150" windowWidth="22995" windowHeight="9525"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPORT_TRIAL" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>CUSTOMER_PO</t>
   </si>
@@ -34,29 +53,41 @@
     <t>ORDER TYPE</t>
   </si>
   <si>
-    <t>484040K01000</t>
-  </si>
-  <si>
     <t>SPECIAL</t>
   </si>
   <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BKT SUB-ASSY,SPRING,NO.3RH              </t>
-  </si>
-  <si>
-    <t>TEST_IMPORT_TRIAL</t>
-  </si>
-  <si>
     <t>PART NO</t>
+  </si>
+  <si>
+    <t>BRACKET, RR AXLE HARNESS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIN, RR SHOCK ABSORBER LWR PIVOT </t>
+  </si>
+  <si>
+    <t>PIN, STRAIGHT</t>
+  </si>
+  <si>
+    <t>421730K01000</t>
+  </si>
+  <si>
+    <t>485330K02000</t>
+  </si>
+  <si>
+    <t>90250T000400</t>
+  </si>
+  <si>
+    <t>F3-MKT-P2026-075-8</t>
+  </si>
+  <si>
+    <t>3B</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,6 +228,12 @@
       <color theme="1"/>
       <name val="Microsoft Sans Serif"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="34">
@@ -561,11 +598,27 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="18" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -619,14 +672,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -664,7 +720,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -736,7 +792,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -909,25 +965,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G141"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G140"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.08984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="33.54296875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="16.90625" style="1" customWidth="1"/>
     <col min="7" max="7" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -945,447 +1001,477 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="8">
+        <v>20</v>
+      </c>
+      <c r="F2" s="8">
+        <v>20260220</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="8">
+        <v>15</v>
+      </c>
+      <c r="F3" s="8">
+        <v>20260220</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="E4" s="8">
+        <v>15</v>
+      </c>
+      <c r="F4" s="8">
+        <v>20260220</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2" s="1">
-        <v>20170807</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F5"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C16" s="2"/>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C17" s="2"/>
     </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C18" s="2"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C19" s="2"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C20" s="2"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C21" s="2"/>
     </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C22" s="2"/>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C23" s="2"/>
     </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C26" s="2"/>
     </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C27" s="2"/>
     </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C28" s="2"/>
     </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C29" s="2"/>
     </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C31" s="2"/>
     </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C32" s="2"/>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C33" s="2"/>
     </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C34" s="2"/>
     </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C35" s="2"/>
     </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C36" s="2"/>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C37" s="2"/>
     </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C38" s="2"/>
     </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C39" s="2"/>
     </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C40" s="2"/>
     </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C41" s="2"/>
     </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C42" s="2"/>
     </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C43" s="2"/>
     </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C47" s="2"/>
     </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C48" s="2"/>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C49" s="2"/>
     </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C50" s="2"/>
     </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C51" s="2"/>
     </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C52" s="2"/>
     </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C53" s="2"/>
     </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C54" s="2"/>
     </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C55" s="2"/>
     </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C56" s="2"/>
     </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C57" s="2"/>
     </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C58" s="2"/>
     </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C59" s="2"/>
     </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C60" s="2"/>
     </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C61" s="2"/>
     </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C62" s="2"/>
     </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C63" s="2"/>
     </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C64" s="2"/>
     </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C65" s="2"/>
     </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C66" s="2"/>
     </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C67" s="2"/>
     </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C68" s="2"/>
     </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C69" s="2"/>
     </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C70" s="2"/>
     </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C71" s="2"/>
     </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C72" s="2"/>
     </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C73" s="2"/>
     </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C74" s="2"/>
     </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C75" s="2"/>
     </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C76" s="2"/>
     </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C77" s="2"/>
     </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C78" s="2"/>
     </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C79" s="2"/>
     </row>
-    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C80" s="2"/>
     </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C81" s="2"/>
     </row>
-    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C82" s="2"/>
     </row>
-    <row r="83" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C83" s="2"/>
     </row>
-    <row r="84" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C84" s="2"/>
     </row>
-    <row r="85" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C85" s="2"/>
     </row>
-    <row r="86" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C86" s="2"/>
     </row>
-    <row r="87" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C87" s="2"/>
     </row>
-    <row r="88" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C88" s="2"/>
     </row>
-    <row r="89" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C89" s="2"/>
     </row>
-    <row r="90" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C90" s="2"/>
     </row>
-    <row r="91" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C91" s="2"/>
     </row>
-    <row r="92" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C92" s="2"/>
     </row>
-    <row r="93" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C93" s="2"/>
     </row>
-    <row r="94" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C94" s="2"/>
     </row>
-    <row r="95" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C95" s="2"/>
     </row>
-    <row r="96" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C96" s="2"/>
     </row>
-    <row r="97" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C97" s="2"/>
     </row>
-    <row r="98" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C98" s="2"/>
     </row>
-    <row r="99" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C99" s="2"/>
     </row>
-    <row r="100" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C100" s="2"/>
     </row>
-    <row r="101" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C101" s="2"/>
     </row>
-    <row r="102" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C102" s="2"/>
     </row>
-    <row r="103" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C103" s="2"/>
     </row>
-    <row r="104" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C104" s="2"/>
     </row>
-    <row r="105" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C105" s="2"/>
     </row>
-    <row r="106" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C106" s="2"/>
     </row>
-    <row r="107" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C107" s="2"/>
     </row>
-    <row r="108" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C108" s="2"/>
     </row>
-    <row r="109" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C115" s="2"/>
     </row>
-    <row r="116" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C116" s="2"/>
     </row>
-    <row r="117" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C117" s="2"/>
     </row>
-    <row r="118" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C118" s="2"/>
     </row>
-    <row r="119" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C119" s="2"/>
     </row>
-    <row r="120" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C120" s="2"/>
     </row>
-    <row r="121" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C121" s="2"/>
     </row>
-    <row r="122" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C122" s="2"/>
     </row>
-    <row r="123" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C123" s="2"/>
     </row>
-    <row r="124" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C124" s="2"/>
     </row>
-    <row r="125" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C125" s="2"/>
     </row>
-    <row r="126" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C126" s="2"/>
     </row>
-    <row r="127" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C127" s="2"/>
     </row>
-    <row r="128" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C128" s="2"/>
     </row>
-    <row r="129" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C129" s="2"/>
     </row>
-    <row r="130" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C130" s="2"/>
     </row>
-    <row r="131" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C131" s="2"/>
     </row>
-    <row r="132" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C132" s="2"/>
     </row>
-    <row r="133" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C133" s="2"/>
     </row>
-    <row r="134" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C134" s="2"/>
     </row>
-    <row r="135" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C135" s="2"/>
     </row>
-    <row r="136" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C136" s="2"/>
     </row>
-    <row r="137" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C137" s="2"/>
     </row>
-    <row r="138" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C138" s="2"/>
     </row>
-    <row r="139" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C139" s="2"/>
     </row>
-    <row r="140" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="3:3" x14ac:dyDescent="0.35">
       <c r="C140" s="2"/>
     </row>
-    <row r="141" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C141" s="2"/>
-    </row>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>